<commit_message>
KPI de salud, simuladores, Tableau igual a Power BI y README con capturas
Pagina Que mide cada KPI en los cuatro tableros, simulador de matronas en colegios (ITS y embarazo), Tableau con las mismas paginas, capturas nuevas, logo con registro y fondo.
</commit_message>
<xml_diff>
--- a/dashboard-ajuar-chile-crece-contigo/Ajuar_PARN_BaseDatos.xlsx
+++ b/dashboard-ajuar-chile-crece-contigo/Ajuar_PARN_BaseDatos.xlsx
@@ -14,7 +14,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contenido" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hallazgos" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPILargo" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -67,11 +69,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -235,7 +240,39 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Fuentes" displayName="Fuentes" ref="A1:C9" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="KPI" displayName="KPI" ref="A1:I9" headerRowCount="1">
+  <autoFilter ref="A1:I9"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="Orden"/>
+    <tableColumn id="2" name="Area"/>
+    <tableColumn id="3" name="KPI"/>
+    <tableColumn id="4" name="Valor"/>
+    <tableColumn id="5" name="Formula"/>
+    <tableColumn id="6" name="QueMide"/>
+    <tableColumn id="7" name="PorQue"/>
+    <tableColumn id="8" name="Meta"/>
+    <tableColumn id="9" name="FuenteID"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="KPILargo" displayName="KPILargo" ref="A1:E57" headerRowCount="1">
+  <autoFilter ref="A1:E57"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="OrdenKPI"/>
+    <tableColumn id="2" name="KPI"/>
+    <tableColumn id="3" name="OrdenCampo"/>
+    <tableColumn id="4" name="Campo"/>
+    <tableColumn id="5" name="Valor"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Fuentes" displayName="Fuentes" ref="A1:C9" headerRowCount="1">
   <autoFilter ref="A1:C9"/>
   <tableColumns count="3">
     <tableColumn id="1" name="FuenteID"/>
@@ -574,6 +611,181 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>FuenteID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Referencia</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Chile Crece Contigo: Programa de Apoyo al Recién Nacido (contenido, requisitos y entrega).</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.crececontigo.gob.cl/beneficios/programa-de-apoyo-al-recien-nacido/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Chile Crece Contigo: requisitos para recibir el set de implementos del PARN.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.crececontigo.gob.cl/faqs/cuales-son-los-requisitos-para-recibir-el-set-de-implementos-del-parn/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DIPRES, Ministerio de Hacienda: Evaluación focalizada de ámbito del Programa de Apoyo al Recién Nacido, informe final (marzo 2024; período 2010–2022).</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://www.dipres.gob.cl/597/articles-341569_informe_final.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MINSAL: Programa de Apoyo al Recién Nacido(a), Informe Glosa 04 año 2018.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.minsal.cl/wp-content/uploads/2019/03/Glosa-4_PARN_2018.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Cenabast: Minsal y Cenabast entregan detalles del nuevo set de implementos para el recién nacido (2016).</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.cenabast.cl/minsal-y-cenabast-entregan-detalles-para-el-nuevo-set-de-implementos-para-el-recien-nacidoa/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BioBioChile: recorte al Ajuar para recién nacidos, qué incluye y por qué se redujo su presupuesto (30-04-2026).</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://www.biobiochile.cl/noticias/bbcl-explica/bbcl-explica-notas/2026/04/30/recorte-al-ajuar-para-recien-nacidos-que-incluye-y-por-que-el-gobierno-redujo-su-presupuesto.shtml</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>La Tercera: qué contiene el ajuar de recién nacidos que el gobierno aclaró que no se dejará de entregar (2026).</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://www.latercera.com/nacional/noticia/que-contiene-el-ajuar-de-recien-nacidos-que-el-gobierno-aclaro-que-no-se-dejara-de-entregar-pese-a-recortes-presupuestarios/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>INE: Anuarios de Estadísticas Vitales (nacidos vivos en Chile).</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://www.ine.gob.cl/estadisticas/sociales/demografia-y-vitales/nacimientos-matrimonios-y-defunciones</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2050,164 +2262,1763 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>Orden</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>QueMide</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>PorQue</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
           <t>FuenteID</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Entregas y cobertura</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Cobertura del set</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>97–99% (2019–2022)</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Sets entregados ÷ nacidos vivos en la red pública × 100</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Cuántas guaguas que tienen derecho al ajuar lo reciben</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Mide si el programa llega a toda su población objetivo</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Entregas y cobertura</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Proporción de nacidos vivos del país con set</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>60,1% (2022)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Sets entregados ÷ nacidos vivos en Chile × 100</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Alcance del programa en todo el país</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>El resto nace en clínicas privadas, que no entregan el set</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>P3;P8</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Entregas y cobertura</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Sets entregados</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>113.858 (2022)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Número de sets entregados en el año</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Producción del programa</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Se ajusta a la natalidad: bajó de 141.883 (2018) a 100.977 (2021)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Presupuesto</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Ejecución presupuestaria</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>85% (2018)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Gasto ejecutado ÷ presupuesto asignado × 100</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Qué parte del dinero asignado se usó</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Un valor bajo puede indicar compras atrasadas o sobrestock</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Cercano a 100%</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Presupuesto</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Costo unitario por set</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>$67.480 neto (2018)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Costo total de compra y distribución ÷ sets</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Cuánto cuesta cada ajuar</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Permite evaluar eficiencia y comparar licitaciones</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Presupuesto</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Variación del presupuesto</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>−10,5% (2026)</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>(Presupuesto del año − año anterior) ÷ año anterior × 100</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Cuánto cambia el financiamiento</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Se justificó por la baja de natalidad y el stock alto</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Garantizar la entrega</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>P6;P7</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Cadena logística</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Puntos de entrega</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>137 maternidades</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Número de maternidades públicas que entregan el set</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Acceso territorial al programa</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Más puntos de entrega = más familias lo reciben al alta</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Todas las maternidades públicas</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Cadena logística</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Participación en el taller educativo</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>95,5% (2018)</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Madres que asistieron al taller ÷ madres que recibieron el set × 100</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Si la familia aprende a usar cada artículo</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>El taller de la matrona es el paso que da sentido al ajuar: sueño seguro, lactancia y apego</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>OrdenKPI</t>
+        </is>
+      </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Referencia</t>
+          <t>KPI</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>URL</t>
+          <t>OrdenCampo</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Valor</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Chile Crece Contigo: Programa de Apoyo al Recién Nacido (contenido, requisitos y entrega).</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>https://www.crececontigo.gob.cl/beneficios/programa-de-apoyo-al-recien-nacido/</t>
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Cobertura del set</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Valor en Chile</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>97–99% (2019–2022)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Chile Crece Contigo: requisitos para recibir el set de implementos del PARN.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>https://www.crececontigo.gob.cl/faqs/cuales-son-los-requisitos-para-recibir-el-set-de-implementos-del-parn/</t>
+      <c r="A3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Cobertura del set</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Cómo se calcula</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Sets entregados ÷ nacidos vivos en la red pública × 100</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Cobertura del set</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Qué evalúa</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Cuántas guaguas que tienen derecho al ajuar lo reciben</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Cobertura del set</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Por qué importa</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Mide si el programa llega a toda su población objetivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Cobertura del set</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Meta o referencia</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Cobertura del set</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Página del tablero</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Entregas y cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Cobertura del set</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>DIPRES, Ministerio de Hacienda: Evaluación focalizada de ámbito del Programa de Apoyo al Recién Nacido, informe final (marzo 2024; período 2010–2022).</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>https://www.dipres.gob.cl/597/articles-341569_informe_final.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Proporción de nacidos vivos del país con set</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Valor en Chile</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>60,1% (2022)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Proporción de nacidos vivos del país con set</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Cómo se calcula</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Sets entregados ÷ nacidos vivos en Chile × 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Proporción de nacidos vivos del país con set</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Qué evalúa</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Alcance del programa en todo el país</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Proporción de nacidos vivos del país con set</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Por qué importa</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>El resto nace en clínicas privadas, que no entregan el set</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Proporción de nacidos vivos del país con set</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Meta o referencia</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Proporción de nacidos vivos del país con set</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Página del tablero</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Entregas y cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Proporción de nacidos vivos del país con set</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>P3;P8</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Sets entregados</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Valor en Chile</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>113.858 (2022)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Sets entregados</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Cómo se calcula</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Número de sets entregados en el año</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Sets entregados</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Qué evalúa</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Producción del programa</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Sets entregados</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Por qué importa</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Se ajusta a la natalidad: bajó de 141.883 (2018) a 100.977 (2021)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Sets entregados</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Meta o referencia</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Sets entregados</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Página del tablero</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Entregas y cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Sets entregados</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Ejecución presupuestaria</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Valor en Chile</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>85% (2018)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Ejecución presupuestaria</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Cómo se calcula</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Gasto ejecutado ÷ presupuesto asignado × 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Ejecución presupuestaria</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Qué evalúa</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Qué parte del dinero asignado se usó</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Ejecución presupuestaria</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Por qué importa</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Un valor bajo puede indicar compras atrasadas o sobrestock</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Ejecución presupuestaria</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Meta o referencia</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Cercano a 100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Ejecución presupuestaria</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Página del tablero</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Presupuesto</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Ejecución presupuestaria</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>MINSAL: Programa de Apoyo al Recién Nacido(a), Informe Glosa 04 año 2018.</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>https://www.minsal.cl/wp-content/uploads/2019/03/Glosa-4_PARN_2018.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Cenabast: Minsal y Cenabast entregan detalles del nuevo set de implementos para el recién nacido (2016).</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>https://www.cenabast.cl/minsal-y-cenabast-entregan-detalles-para-el-nuevo-set-de-implementos-para-el-recien-nacidoa/</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>P6</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>BioBioChile: recorte al Ajuar para recién nacidos, qué incluye y por qué se redujo su presupuesto (30-04-2026).</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>https://www.biobiochile.cl/noticias/bbcl-explica/bbcl-explica-notas/2026/04/30/recorte-al-ajuar-para-recien-nacidos-que-incluye-y-por-que-el-gobierno-redujo-su-presupuesto.shtml</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>La Tercera: qué contiene el ajuar de recién nacidos que el gobierno aclaró que no se dejará de entregar (2026).</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>https://www.latercera.com/nacional/noticia/que-contiene-el-ajuar-de-recien-nacidos-que-el-gobierno-aclaro-que-no-se-dejara-de-entregar-pese-a-recortes-presupuestarios/</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>INE: Anuarios de Estadísticas Vitales (nacidos vivos en Chile).</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>https://www.ine.gob.cl/estadisticas/sociales/demografia-y-vitales/nacimientos-matrimonios-y-defunciones</t>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Costo unitario por set</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Valor en Chile</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>$67.480 neto (2018)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Costo unitario por set</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Cómo se calcula</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Costo total de compra y distribución ÷ sets</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Costo unitario por set</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Qué evalúa</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Cuánto cuesta cada ajuar</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Costo unitario por set</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Por qué importa</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Permite evaluar eficiencia y comparar licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Costo unitario por set</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Meta o referencia</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Costo unitario por set</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Página del tablero</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Presupuesto</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Costo unitario por set</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Variación del presupuesto</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Valor en Chile</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>−10,5% (2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Variación del presupuesto</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Cómo se calcula</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>(Presupuesto del año − año anterior) ÷ año anterior × 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Variación del presupuesto</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Qué evalúa</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Cuánto cambia el financiamiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Variación del presupuesto</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Por qué importa</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Se justificó por la baja de natalidad y el stock alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Variación del presupuesto</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Meta o referencia</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Garantizar la entrega</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Variación del presupuesto</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Página del tablero</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Presupuesto</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Variación del presupuesto</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>P6;P7</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Puntos de entrega</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Valor en Chile</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>137 maternidades</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Puntos de entrega</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Cómo se calcula</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Número de maternidades públicas que entregan el set</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Puntos de entrega</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Qué evalúa</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Acceso territorial al programa</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Puntos de entrega</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Por qué importa</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Más puntos de entrega = más familias lo reciben al alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Puntos de entrega</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Meta o referencia</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Todas las maternidades públicas</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Puntos de entrega</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Página del tablero</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Cadena logística</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Puntos de entrega</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Participación en el taller educativo</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Valor en Chile</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>95,5% (2018)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Participación en el taller educativo</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Cómo se calcula</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Madres que asistieron al taller ÷ madres que recibieron el set × 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Participación en el taller educativo</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Qué evalúa</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Si la familia aprende a usar cada artículo</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Participación en el taller educativo</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Por qué importa</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>El taller de la matrona es el paso que da sentido al ajuar: sueño seguro, lactancia y apego</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Participación en el taller educativo</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Meta o referencia</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Participación en el taller educativo</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Página del tablero</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Cadena logística</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Participación en el taller educativo</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>P4</t>
         </is>
       </c>
     </row>

</xml_diff>